<commit_message>
fix(ci/cd): complete end-to-end recovery, executive reporting, Security SAST, Next.js static export & GitHub Pages deployment
</commit_message>
<xml_diff>
--- a/SecurityTest/reports/web-security-findings.xlsx
+++ b/SecurityTest/reports/web-security-findings.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M12"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
@@ -474,7 +474,7 @@
       <c r="E2" t="str">
         <v>DashboardLayout</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="str">
         <v>19</v>
       </c>
       <c r="G2" t="str">
@@ -510,13 +510,13 @@
         <v>Authorization / Client-Side Auth Guard</v>
       </c>
       <c r="D3" t="str">
-        <v>/src/app/(dashboard)/trips/[id]/page.tsx</v>
+        <v>/src/app/(dashboard)/trips/[id]/TripDetailClient.tsx</v>
       </c>
       <c r="E3" t="str">
         <v>DashboardLayout</v>
       </c>
-      <c r="F3">
-        <v>63</v>
+      <c r="F3" t="str">
+        <v>61</v>
       </c>
       <c r="G3" t="str">
         <v>Route protection is implemented client-side only using useEffect. This creates a brief window where protected content may flash before redirect.</v>
@@ -537,7 +537,7 @@
         <v>A01 - Broken Access Control</v>
       </c>
       <c r="M3" t="str">
-        <v>useEffect-based auth guard in \src\app\(dashboard)\trips\[id]\page.tsx</v>
+        <v>useEffect-based auth guard in \src\app\(dashboard)\trips\[id]\TripDetailClient.tsx</v>
       </c>
     </row>
     <row r="4">
@@ -556,7 +556,7 @@
       <c r="E4" t="str">
         <v>headers()</v>
       </c>
-      <c r="F4">
+      <c r="F4" t="str">
         <v>39</v>
       </c>
       <c r="G4" t="str">
@@ -597,7 +597,7 @@
       <c r="E5" t="str">
         <v>N/A</v>
       </c>
-      <c r="F5">
+      <c r="F5" t="str">
         <v>394</v>
       </c>
       <c r="G5" t="str">
@@ -638,7 +638,7 @@
       <c r="E6" t="str">
         <v>N/A</v>
       </c>
-      <c r="F6">
+      <c r="F6" t="str">
         <v>413</v>
       </c>
       <c r="G6" t="str">
@@ -668,10 +668,10 @@
         <v>WEB-0006</v>
       </c>
       <c r="B7" t="str">
-        <v>MODERATE</v>
+        <v>MEDIUM</v>
       </c>
       <c r="C7" t="str">
-        <v>Dependencies / next</v>
+        <v>Dependencies / brace-expansion</v>
       </c>
       <c r="D7" t="str">
         <v>/package.json</v>
@@ -679,17 +679,17 @@
       <c r="E7" t="str">
         <v>N/A</v>
       </c>
-      <c r="F7">
+      <c r="F7" t="str">
         <v>1</v>
       </c>
       <c r="G7" t="str">
-        <v>npm audit found MODERATE severity vulnerability in next.</v>
+        <v>npm audit advisory for dev/build dependency brace-expansion.</v>
       </c>
       <c r="H7" t="str">
-        <v>next version has a known security vulnerability.</v>
+        <v>brace-expansion version has a known security advisory.</v>
       </c>
       <c r="I7" t="str">
-        <v>Dependency vulnerability in next may be exploitable depending on usage.</v>
+        <v>Build-time dependency advisory in brace-expansion.</v>
       </c>
       <c r="J7" t="str">
         <v>Run 'npm audit fix' to resolve.</v>
@@ -701,7 +701,7 @@
         <v>A06 - Vulnerable and Outdated Components</v>
       </c>
       <c r="M7" t="str">
-        <v>next: moderate</v>
+        <v>brace-expansion: high</v>
       </c>
     </row>
     <row r="8">
@@ -709,10 +709,10 @@
         <v>WEB-0007</v>
       </c>
       <c r="B8" t="str">
-        <v>MODERATE</v>
+        <v>MEDIUM</v>
       </c>
       <c r="C8" t="str">
-        <v>Dependencies / postcss</v>
+        <v>Dependencies / js-yaml</v>
       </c>
       <c r="D8" t="str">
         <v>/package.json</v>
@@ -720,17 +720,17 @@
       <c r="E8" t="str">
         <v>N/A</v>
       </c>
-      <c r="F8">
+      <c r="F8" t="str">
         <v>1</v>
       </c>
       <c r="G8" t="str">
-        <v>npm audit found MODERATE severity vulnerability in postcss.</v>
+        <v>npm audit advisory for dev/build dependency js-yaml.</v>
       </c>
       <c r="H8" t="str">
-        <v>postcss version has a known security vulnerability.</v>
+        <v>js-yaml version has a known security advisory.</v>
       </c>
       <c r="I8" t="str">
-        <v>Dependency vulnerability in postcss may be exploitable depending on usage.</v>
+        <v>Build-time dependency advisory in js-yaml.</v>
       </c>
       <c r="J8" t="str">
         <v>Run 'npm audit fix' to resolve.</v>
@@ -742,19 +742,183 @@
         <v>A06 - Vulnerable and Outdated Components</v>
       </c>
       <c r="M8" t="str">
+        <v>js-yaml: high</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>WEB-0008</v>
+      </c>
+      <c r="B9" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Dependencies / next</v>
+      </c>
+      <c r="D9" t="str">
+        <v>/package.json</v>
+      </c>
+      <c r="E9" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F9" t="str">
+        <v>1</v>
+      </c>
+      <c r="G9" t="str">
+        <v>npm audit advisory for dev/build dependency next.</v>
+      </c>
+      <c r="H9" t="str">
+        <v>next version has a known security advisory.</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Build-time dependency advisory in next.</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Run 'npm audit fix' to resolve.</v>
+      </c>
+      <c r="K9" t="str">
+        <v>CWE-1104</v>
+      </c>
+      <c r="L9" t="str">
+        <v>A06 - Vulnerable and Outdated Components</v>
+      </c>
+      <c r="M9" t="str">
+        <v>next: high</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>WEB-0009</v>
+      </c>
+      <c r="B10" t="str">
+        <v>MODERATE</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Dependencies / postcss</v>
+      </c>
+      <c r="D10" t="str">
+        <v>/package.json</v>
+      </c>
+      <c r="E10" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F10" t="str">
+        <v>1</v>
+      </c>
+      <c r="G10" t="str">
+        <v>npm audit advisory for dev/build dependency postcss.</v>
+      </c>
+      <c r="H10" t="str">
+        <v>postcss version has a known security advisory.</v>
+      </c>
+      <c r="I10" t="str">
+        <v>Build-time dependency advisory in postcss.</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Run 'npm audit fix' to resolve.</v>
+      </c>
+      <c r="K10" t="str">
+        <v>CWE-1104</v>
+      </c>
+      <c r="L10" t="str">
+        <v>A06 - Vulnerable and Outdated Components</v>
+      </c>
+      <c r="M10" t="str">
         <v>postcss: moderate</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>WEB-0010</v>
+      </c>
+      <c r="B11" t="str">
+        <v>MODERATE</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Dependencies / protobufjs</v>
+      </c>
+      <c r="D11" t="str">
+        <v>/package.json</v>
+      </c>
+      <c r="E11" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F11" t="str">
+        <v>1</v>
+      </c>
+      <c r="G11" t="str">
+        <v>npm audit advisory for dev/build dependency protobufjs.</v>
+      </c>
+      <c r="H11" t="str">
+        <v>protobufjs version has a known security advisory.</v>
+      </c>
+      <c r="I11" t="str">
+        <v>Build-time dependency advisory in protobufjs.</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Run 'npm audit fix' to resolve.</v>
+      </c>
+      <c r="K11" t="str">
+        <v>CWE-1104</v>
+      </c>
+      <c r="L11" t="str">
+        <v>A06 - Vulnerable and Outdated Components</v>
+      </c>
+      <c r="M11" t="str">
+        <v>protobufjs: moderate</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>WEB-0011</v>
+      </c>
+      <c r="B12" t="str">
+        <v>MEDIUM</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Dependencies / sharp</v>
+      </c>
+      <c r="D12" t="str">
+        <v>/package.json</v>
+      </c>
+      <c r="E12" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="F12" t="str">
+        <v>1</v>
+      </c>
+      <c r="G12" t="str">
+        <v>npm audit advisory for dev/build dependency sharp.</v>
+      </c>
+      <c r="H12" t="str">
+        <v>sharp version has a known security advisory.</v>
+      </c>
+      <c r="I12" t="str">
+        <v>Build-time dependency advisory in sharp.</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Run 'npm audit fix' to resolve.</v>
+      </c>
+      <c r="K12" t="str">
+        <v>CWE-1104</v>
+      </c>
+      <c r="L12" t="str">
+        <v>A06 - Vulnerable and Outdated Components</v>
+      </c>
+      <c r="M12" t="str">
+        <v>sharp: high</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F15"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="20.83203125" customWidth="1"/>
@@ -826,167 +990,247 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>next</v>
+        <v>brace-expansion</v>
       </c>
       <c r="B4" t="str">
-        <v>9.3.4-canary.0 - 16.3.0-canary.5</v>
+        <v>&lt;1.1.16 || &gt;=3.0.0 &lt;5.0.7</v>
       </c>
       <c r="C4" t="str">
         <v>Fix available</v>
       </c>
       <c r="D4" t="str">
-        <v>MODERATE</v>
+        <v>HIGH</v>
       </c>
       <c r="E4" t="str">
-        <v>next: postcss</v>
+        <v>brace-expansion: brace-expansion: DoS via exponential-time expansion of consecutive non-expanding {} groups, brace-expansion: DoS via exponential-time expansion of consecutive non-expanding {} groups</v>
       </c>
       <c r="F4" t="str">
-        <v>Run 'npm audit fix' or update next to the fixed version.</v>
+        <v>Run 'npm audit fix' or update brace-expansion to the fixed version.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>postcss</v>
+        <v>js-yaml</v>
       </c>
       <c r="B5" t="str">
-        <v>&lt;8.5.10</v>
+        <v>4.0.0 - 4.2.0</v>
       </c>
       <c r="C5" t="str">
         <v>Fix available</v>
       </c>
       <c r="D5" t="str">
-        <v>MODERATE</v>
+        <v>HIGH</v>
       </c>
       <c r="E5" t="str">
-        <v>postcss: PostCSS has XSS via Unescaped &lt;/style&gt; in its CSS Stringify Output</v>
+        <v>js-yaml: js-yaml: YAML merge-key chains can force quadratic CPU consumption</v>
       </c>
       <c r="F5" t="str">
-        <v>Run 'npm audit fix' or update postcss to the fixed version.</v>
+        <v>Run 'npm audit fix' or update js-yaml to the fixed version.</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>@tanstack/react-query</v>
+        <v>next</v>
       </c>
       <c r="B6" t="str">
-        <v>^5.101.0</v>
+        <v>9.3.4-canary.0 - 16.3.0-preview.7</v>
       </c>
       <c r="C6" t="str">
-        <v>5.x</v>
+        <v>Fix available</v>
       </c>
       <c r="D6" t="str">
-        <v>INFO</v>
+        <v>HIGH</v>
       </c>
       <c r="E6" t="str">
-        <v>Monitor for updates</v>
+        <v>next: postcss, sharp</v>
       </c>
       <c r="F6" t="str">
-        <v>Run 'npm audit' and update @tanstack/react-query regularly</v>
+        <v>Run 'npm audit fix' or update next to the fixed version.</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>framer-motion</v>
+        <v>postcss</v>
       </c>
       <c r="B7" t="str">
-        <v>^12.40.0</v>
+        <v>&lt;8.5.10</v>
       </c>
       <c r="C7" t="str">
-        <v>12.x</v>
+        <v>Fix available</v>
       </c>
       <c r="D7" t="str">
-        <v>INFO</v>
+        <v>MODERATE</v>
       </c>
       <c r="E7" t="str">
-        <v>Monitor for updates</v>
+        <v>postcss: PostCSS has XSS via Unescaped &lt;/style&gt; in its CSS Stringify Output</v>
       </c>
       <c r="F7" t="str">
-        <v>Run 'npm audit' and update framer-motion regularly</v>
+        <v>Run 'npm audit fix' or update postcss to the fixed version.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>leaflet</v>
+        <v>protobufjs</v>
       </c>
       <c r="B8" t="str">
-        <v>^1.9.4</v>
+        <v>7.5.0 - 7.6.4</v>
       </c>
       <c r="C8" t="str">
-        <v>1.9.x</v>
+        <v>Fix available</v>
       </c>
       <c r="D8" t="str">
-        <v>INFO</v>
+        <v>MODERATE</v>
       </c>
       <c r="E8" t="str">
-        <v>No known critical CVEs in current version</v>
+        <v>protobufjs: protobufjs: Denial of Service via infinite loop in .proto option parsing</v>
       </c>
       <c r="F8" t="str">
-        <v>Run 'npm audit' and update leaflet regularly</v>
+        <v>Run 'npm audit fix' or update protobufjs to the fixed version.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>react</v>
+        <v>sharp</v>
       </c>
       <c r="B9" t="str">
-        <v>19.2.4</v>
+        <v>&lt;0.35.0</v>
       </c>
       <c r="C9" t="str">
-        <v>19.x</v>
+        <v>Fix available</v>
       </c>
       <c r="D9" t="str">
-        <v>INFO</v>
+        <v>HIGH</v>
       </c>
       <c r="E9" t="str">
-        <v>Current, monitor for patches</v>
+        <v>sharp: sharp inherited vulnerabilities in libvips: CVE-2026-33327, CVE-2026-33328, CVE-2026-35590, CVE-2026-35591</v>
       </c>
       <c r="F9" t="str">
-        <v>Run 'npm audit' and update react regularly</v>
+        <v>Run 'npm audit fix' or update sharp to the fixed version.</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>zod</v>
+        <v>@tanstack/react-query</v>
       </c>
       <c r="B10" t="str">
-        <v>^4.4.3</v>
+        <v>^5.101.0</v>
       </c>
       <c r="C10" t="str">
-        <v>4.x</v>
+        <v>5.x</v>
       </c>
       <c r="D10" t="str">
         <v>INFO</v>
       </c>
       <c r="E10" t="str">
-        <v>Schema validation library, keep updated</v>
+        <v>Monitor for updates</v>
       </c>
       <c r="F10" t="str">
-        <v>Run 'npm audit' and update zod regularly</v>
+        <v>Run 'npm audit' and update @tanstack/react-query regularly</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>typescript</v>
+        <v>framer-motion</v>
       </c>
       <c r="B11" t="str">
-        <v>^5</v>
+        <v>^12.40.0</v>
       </c>
       <c r="C11" t="str">
-        <v>5.x</v>
+        <v>12.x</v>
       </c>
       <c r="D11" t="str">
         <v>INFO</v>
       </c>
       <c r="E11" t="str">
+        <v>Monitor for updates</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Run 'npm audit' and update framer-motion regularly</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>leaflet</v>
+      </c>
+      <c r="B12" t="str">
+        <v>^1.9.4</v>
+      </c>
+      <c r="C12" t="str">
+        <v>1.9.x</v>
+      </c>
+      <c r="D12" t="str">
+        <v>INFO</v>
+      </c>
+      <c r="E12" t="str">
+        <v>No known critical CVEs in current version</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Run 'npm audit' and update leaflet regularly</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>react</v>
+      </c>
+      <c r="B13" t="str">
+        <v>19.2.4</v>
+      </c>
+      <c r="C13" t="str">
+        <v>19.x</v>
+      </c>
+      <c r="D13" t="str">
+        <v>INFO</v>
+      </c>
+      <c r="E13" t="str">
         <v>Current, monitor for patches</v>
       </c>
-      <c r="F11" t="str">
+      <c r="F13" t="str">
+        <v>Run 'npm audit' and update react regularly</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>zod</v>
+      </c>
+      <c r="B14" t="str">
+        <v>^4.4.3</v>
+      </c>
+      <c r="C14" t="str">
+        <v>4.x</v>
+      </c>
+      <c r="D14" t="str">
+        <v>INFO</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Schema validation library, keep updated</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Run 'npm audit' and update zod regularly</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>typescript</v>
+      </c>
+      <c r="B15" t="str">
+        <v>^5</v>
+      </c>
+      <c r="C15" t="str">
+        <v>5.x</v>
+      </c>
+      <c r="D15" t="str">
+        <v>INFO</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Current, monitor for patches</v>
+      </c>
+      <c r="F15" t="str">
         <v>Run 'npm audit' and update typescript regularly</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F15"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1016,7 +1260,7 @@
         <v>Generated</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-07-19T17:28:16.402Z</v>
+        <v>2026-07-22T16:57:17.726Z</v>
       </c>
     </row>
     <row r="4">
@@ -1092,13 +1336,13 @@
         <v>MEDIUM</v>
       </c>
       <c r="B11">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="C11">
         <v>4</v>
       </c>
       <c r="D11">
-        <v>20</v>
+        <v>36</v>
       </c>
     </row>
     <row r="12">
@@ -1134,13 +1378,13 @@
         <v>TOTAL</v>
       </c>
       <c r="B14">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C14" t="str">
         <v/>
       </c>
       <c r="D14">
-        <v>20</v>
+        <v>36</v>
       </c>
     </row>
     <row r="15">
@@ -1153,7 +1397,7 @@
         <v>Overall Risk Level</v>
       </c>
       <c r="B16" t="str">
-        <v>LOW RISK</v>
+        <v>MEDIUM RISK</v>
       </c>
     </row>
     <row r="17">
@@ -1161,7 +1405,7 @@
         <v>Risk Score</v>
       </c>
       <c r="B17" t="str">
-        <v>20/100</v>
+        <v>36/100</v>
       </c>
     </row>
     <row r="18">
@@ -1184,15 +1428,15 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Authorization</v>
+        <v>Dependencies</v>
       </c>
       <c r="B21">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Authentication</v>
+        <v>Authorization</v>
       </c>
       <c r="B22">
         <v>2</v>
@@ -1200,7 +1444,7 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Dependencies</v>
+        <v>Authentication</v>
       </c>
       <c r="B23">
         <v>2</v>

</xml_diff>